<commit_message>
Atualização do arquivo inventario_tratado.xlsx
</commit_message>
<xml_diff>
--- a/ingest/inventario_tratado.xlsx
+++ b/ingest/inventario_tratado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e0da82f14d1f41d/Documentos/PowerBi do projeto de BigData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{E904733D-3307-4C8D-9C96-5FAF6DB0D327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4081ED2C-F04C-40D2-BAE7-305AF81296DF}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{E904733D-3307-4C8D-9C96-5FAF6DB0D327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{477E2939-C215-4141-A414-05E41D70EB95}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{83CE71C9-A43E-4812-B57A-46D4875B135E}"/>
   </bookViews>
@@ -3100,6 +3100,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -3431,7 +3435,7 @@
     <col min="8" max="8" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.88671875" style="1" customWidth="1"/>
     <col min="12" max="12" width="14" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.44140625" style="1" bestFit="1" customWidth="1"/>

</xml_diff>